<commit_message>
Prepare secure test infrastructure, Allure reporting and thesis documentation
</commit_message>
<xml_diff>
--- a/docs/test-documentation/Test_Matrix_updated.xlsx
+++ b/docs/test-documentation/Test_Matrix_updated.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Матрица" sheetId="1" r:id="Rfef2258963904e33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Матрица" sheetId="1" r:id="R8023718d6f2e458e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Первоначальный план" sheetId="2" r:id="R3e118bc75ab6401a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45,7 +46,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -73,6 +74,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -81,13 +85,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TableTestMatrix" displayName="TableTestMatrix" ref="A1:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TableTestMatrix" displayName="TableTestMatrix" ref="A1:H9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID требования"/>
     <x:tableColumn id="2" name="Функция"/>
     <x:tableColumn id="3" name="UI-кейсы"/>
     <x:tableColumn id="4" name="API-кейсы"/>
     <x:tableColumn id="5" name="Статус покрытия"/>
+    <x:tableColumn id="6" name="Самостоятельных кейсов"/>
+    <x:tableColumn id="7" name="Java-методов"/>
+    <x:tableColumn id="8" name="Выполнений Regression"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="DocMatrix1" displayName="DocMatrix1" ref="A1:H3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="ID требования"/>
+    <x:tableColumn id="2" name="Функция"/>
+    <x:tableColumn id="3" name="UI-кейсы"/>
+    <x:tableColumn id="4" name="API-кейсы"/>
+    <x:tableColumn id="5" name="Статус покрытия"/>
+    <x:tableColumn id="6" name="Самостоятельных кейсов"/>
+    <x:tableColumn id="7" name="Java-методов"/>
+    <x:tableColumn id="8" name="Выполнений Regression"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -288,31 +311,43 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="50" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="65" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="80" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="35" customHeight="1">
-      <x:c r="A1" s="5" t="str">
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="13" t="str">
         <x:v>ID требования</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="13" t="str">
         <x:v>Функция</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="13" t="str">
         <x:v>UI-кейсы</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="13" t="str">
         <x:v>API-кейсы</x:v>
       </x:c>
-      <x:c r="E1" s="5" t="str">
+      <x:c r="E1" s="13" t="str">
         <x:v>Статус покрытия</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="46" customHeight="1">
+      <x:c r="F1" s="13" t="str">
+        <x:v>Самостоятельных кейсов</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>Java-методов</x:v>
+      </x:c>
+      <x:c r="H1" s="13" t="str">
+        <x:v>Выполнений Regression</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="78" customHeight="1">
       <x:c r="A2" s="12" t="str">
         <x:v>REQ-01</x:v>
       </x:c>
@@ -320,16 +355,25 @@
         <x:v>Регистрация и валидация</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>UI-001, UI-002, UI-003, UI-004</x:v>
+        <x:v>UI-001, UI-002, UI-003, UI-004, UI-021, UI-026, UI-027, UI-028, UI-029, UI-030, UI-031, UI-032, UI-040</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
-        <x:v>API-001, API-002, API-003, API-004</x:v>
+        <x:v>API-001, API-002, API-003, API-004, API-021, API-026, API-027, API-028, API-041, API-042, API-043</x:v>
       </x:c>
       <x:c r="E2" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="46" customHeight="1">
+        <x:v>PASS по перечисленным кейсам; 27.10.2026</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G2" s="12" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H2" s="12" t="n">
+        <x:v>47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="78" customHeight="1">
       <x:c r="A3" s="12" t="str">
         <x:v>REQ-02</x:v>
       </x:c>
@@ -337,16 +381,25 @@
         <x:v>Аутентификация и сессия</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>UI-005, UI-006, UI-007, UI-008, UI-009</x:v>
+        <x:v>UI-005, UI-006, UI-007, UI-023, UI-024, UI-025</x:v>
       </x:c>
       <x:c r="D3" s="12" t="str">
-        <x:v>API-020</x:v>
+        <x:v>API-020, API-022, API-023, API-024, API-025, API-036</x:v>
       </x:c>
       <x:c r="E3" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="46" customHeight="1">
+        <x:v>PASS по перечисленным кейсам; 27.10.2026</x:v>
+      </x:c>
+      <x:c r="F3" s="12" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="78" customHeight="1">
       <x:c r="A4" s="12" t="str">
         <x:v>REQ-03</x:v>
       </x:c>
@@ -354,16 +407,25 @@
         <x:v>Просмотр задач</x:v>
       </x:c>
       <x:c r="C4" s="12" t="str">
-        <x:v>UI-010</x:v>
+        <x:v>UI-033, UI-034</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
-        <x:v>API-006, API-007, API-011, API-012</x:v>
+        <x:v>API-006, API-011, API-012</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="46" customHeight="1">
+        <x:v>PASS по перечисленным кейсам; 27.10.2026</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H4" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="78" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>REQ-04</x:v>
       </x:c>
@@ -371,16 +433,25 @@
         <x:v>Создание задач</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>UI-011, UI-012, UI-013, UI-014</x:v>
+        <x:v>UI-011, UI-012, UI-013, UI-014, UI-035, UI-036, UI-037, UI-038</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>API-008, API-009, API-010</x:v>
+        <x:v>API-008, API-009, API-029, API-030, API-031, API-037, API-038, API-039, API-044</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="46" customHeight="1">
+        <x:v>PASS по перечисленным кейсам; 27.10.2026</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="n">
+        <x:v>34</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="78" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>REQ-05</x:v>
       </x:c>
@@ -388,16 +459,25 @@
         <x:v>Изменение задач</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>UI-015, UI-016, UI-017</x:v>
+        <x:v>UI-016</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>API-013, API-014</x:v>
+        <x:v>API-013, API-040</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="46" customHeight="1">
+        <x:v>PASS по перечисленным кейсам; 27.10.2026</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G6" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="n">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="78" customHeight="1">
       <x:c r="A7" s="12" t="str">
         <x:v>REQ-06</x:v>
       </x:c>
@@ -405,16 +485,25 @@
         <x:v>Удаление задач</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>UI-018</x:v>
+        <x:v>UI-018, UI-039</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>API-015, API-016</x:v>
+        <x:v>API-015</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="46" customHeight="1">
+        <x:v>PASS по перечисленным кейсам; 27.10.2026</x:v>
+      </x:c>
+      <x:c r="F7" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G7" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H7" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="78" customHeight="1">
       <x:c r="A8" s="12" t="str">
         <x:v>REQ-07</x:v>
       </x:c>
@@ -422,49 +511,148 @@
         <x:v>Изоляция данных и права</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>UI-019</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>API-017, API-018, API-019</x:v>
+        <x:v>API-017</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="46" customHeight="1">
+        <x:v>PASS по перечисленным кейсам; 27.10.2026</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G8" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="78" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>REQ-08</x:v>
+        <x:v>REQ-10</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Защита пользовательского ввода</x:v>
+        <x:v>Подключение к тестовой PostgreSQL</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>UI-020</x:v>
-      </x:c>
-      <x:c r="D9" s="12" t="str"/>
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="str">
+        <x:v>API-035</x:v>
+      </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="46" customHeight="1">
-      <x:c r="A10" s="12" t="str">
-        <x:v>REQ-09</x:v>
-      </x:c>
-      <x:c r="B10" s="12" t="str">
-        <x:v>Получение CSRF-токена и защита изменяющих запросов</x:v>
-      </x:c>
-      <x:c r="C10" s="12" t="str"/>
-      <x:c r="D10" s="12" t="str">
-        <x:v>API-005, API-010</x:v>
-      </x:c>
-      <x:c r="E10" s="12" t="str">
-        <x:v>Запланировано</x:v>
-      </x:c>
+        <x:v>PASS по перечисленным кейсам; 27.10.2026</x:v>
+      </x:c>
+      <x:c r="F9" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G9" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H9" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" customHeight="1">
+      <x:c r="A10"/>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
+      <x:c r="G10"/>
+      <x:c r="H10"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfebc8287c8d84ef4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0d7fbe282d34996"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="65" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="80" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="38" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>ID требования</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Функция</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>UI-кейсы</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>API-кейсы</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Статус покрытия</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>Самостоятельных кейсов</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>Java-методов</x:v>
+      </x:c>
+      <x:c r="H1" s="13" t="str">
+        <x:v>Выполнений Regression</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="110" customHeight="1">
+      <x:c r="A2" s="12" t="str">
+        <x:v>REQ-08</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="str">
+        <x:v>Защита пользовательского ввода</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="str">
+        <x:v>UI-020</x:v>
+      </x:c>
+      <x:c r="D2" s="12"/>
+      <x:c r="E2" s="12" t="str">
+        <x:v>Вне актуальной матрицы: отдельного реализованного теста нет. CSRF используется при подготовке запросов, это не самостоятельный негативный тест.</x:v>
+      </x:c>
+      <x:c r="F2" s="12"/>
+      <x:c r="G2" s="12"/>
+      <x:c r="H2" s="12"/>
+    </x:row>
+    <x:row r="3" ht="110" customHeight="1">
+      <x:c r="A3" s="12" t="str">
+        <x:v>REQ-09</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="str">
+        <x:v>Получение CSRF-токена и защита изменяющих запросов</x:v>
+      </x:c>
+      <x:c r="C3" s="12"/>
+      <x:c r="D3" s="12" t="str">
+        <x:v>API-005, API-010</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="str">
+        <x:v>Вне актуальной матрицы: отдельного реализованного теста нет. CSRF используется при подготовке запросов, это не самостоятельный негативный тест.</x:v>
+      </x:c>
+      <x:c r="F3" s="12"/>
+      <x:c r="G3" s="12"/>
+      <x:c r="H3" s="12"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c3995763a94452c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>